<commit_message>
Major progress with Propulsion projects, and steering joystick.
Making more stuff!
</commit_message>
<xml_diff>
--- a/10-NX System/!!!Check-In_Check-Out Document.xlsx
+++ b/10-NX System/!!!Check-In_Check-Out Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
   <si>
     <t>System</t>
   </si>
@@ -35,9 +35,6 @@
   </si>
   <si>
     <t>Main Assembly name</t>
-  </si>
-  <si>
-    <t>Jonas</t>
   </si>
   <si>
     <t>Hull</t>
@@ -947,11 +944,9 @@
       <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6" t="s">
-        <v>8</v>
-      </c>
+      <c r="E2" s="6"/>
       <c r="F2" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
@@ -967,11 +962,11 @@
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="13"/>
       <c r="B4" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="15"/>
       <c r="D4" s="16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F4" s="17" t="b">
         <v>0</v>
@@ -981,7 +976,7 @@
       <c r="A5" s="18"/>
       <c r="B5" s="19"/>
       <c r="C5" s="20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D5" s="5"/>
       <c r="F5" s="21" t="b">
@@ -993,7 +988,7 @@
       <c r="B6" s="19"/>
       <c r="C6" s="19"/>
       <c r="D6" s="16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F6" s="21" t="b">
         <v>0</v>
@@ -1004,7 +999,7 @@
       <c r="B7" s="19"/>
       <c r="C7" s="22"/>
       <c r="D7" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F7" s="21" t="b">
         <v>0</v>
@@ -1015,7 +1010,7 @@
       <c r="B8" s="19"/>
       <c r="C8" s="23"/>
       <c r="D8" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8" s="24" t="b">
         <v>0</v>
@@ -1026,7 +1021,7 @@
       <c r="B9" s="19"/>
       <c r="C9" s="23"/>
       <c r="D9" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F9" s="24" t="b">
         <v>0</v>
@@ -1037,7 +1032,7 @@
       <c r="B10" s="19"/>
       <c r="C10" s="23"/>
       <c r="D10" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F10" s="24" t="b">
         <v>0</v>
@@ -1047,7 +1042,7 @@
       <c r="A11" s="18"/>
       <c r="B11" s="19"/>
       <c r="C11" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D11" s="4"/>
       <c r="F11" s="21" t="b">
@@ -1059,7 +1054,7 @@
       <c r="B12" s="19"/>
       <c r="C12" s="19"/>
       <c r="D12" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F12" s="21" t="b">
         <v>0</v>
@@ -1070,7 +1065,7 @@
       <c r="B13" s="19"/>
       <c r="C13" s="22"/>
       <c r="D13" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F13" s="21" t="b">
         <v>0</v>
@@ -1081,7 +1076,7 @@
       <c r="B14" s="19"/>
       <c r="C14" s="19"/>
       <c r="D14" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F14" s="21" t="b">
         <v>0</v>
@@ -1091,7 +1086,7 @@
       <c r="A15" s="18"/>
       <c r="B15" s="19"/>
       <c r="C15" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D15" s="4"/>
       <c r="F15" s="24"/>
@@ -1101,7 +1096,7 @@
       <c r="B16" s="19"/>
       <c r="C16" s="19"/>
       <c r="D16" s="16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F16" s="24"/>
     </row>
@@ -1110,7 +1105,7 @@
       <c r="B17" s="19"/>
       <c r="C17" s="22"/>
       <c r="D17" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F17" s="24"/>
     </row>
@@ -1119,7 +1114,7 @@
       <c r="B18" s="19"/>
       <c r="C18" s="19"/>
       <c r="D18" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E18" s="25"/>
       <c r="F18" s="26" t="b">
@@ -1159,11 +1154,11 @@
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="27"/>
       <c r="B22" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C22" s="15"/>
       <c r="D22" s="28" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E22" s="29"/>
       <c r="F22" s="30" t="b">
@@ -1175,7 +1170,7 @@
       <c r="B23" s="9"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E23" s="11"/>
       <c r="F23" s="26" t="b">
@@ -1187,7 +1182,7 @@
       <c r="B24" s="9"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E24" s="11"/>
       <c r="F24" s="26" t="b">
@@ -1199,7 +1194,7 @@
       <c r="B25" s="9"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E25" s="11"/>
       <c r="F25" s="26" t="b">
@@ -1211,7 +1206,7 @@
       <c r="B26" s="9"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E26" s="11"/>
       <c r="F26" s="26" t="b">
@@ -1232,7 +1227,7 @@
       <c r="A28" s="13"/>
       <c r="B28" s="4"/>
       <c r="C28" s="20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="11"/>
@@ -1245,7 +1240,7 @@
       <c r="B29" s="19"/>
       <c r="C29" s="19"/>
       <c r="D29" s="16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E29" s="32"/>
       <c r="F29" s="7" t="b">
@@ -1257,7 +1252,7 @@
       <c r="B30" s="23"/>
       <c r="C30" s="23"/>
       <c r="D30" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E30" s="32"/>
       <c r="F30" s="34" t="b">
@@ -1269,7 +1264,7 @@
       <c r="B31" s="4"/>
       <c r="C31" s="22"/>
       <c r="D31" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E31" s="35"/>
       <c r="F31" s="17" t="b">
@@ -1281,7 +1276,7 @@
       <c r="B32" s="19"/>
       <c r="C32" s="19"/>
       <c r="D32" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E32" s="32"/>
       <c r="F32" s="7" t="b">
@@ -1302,7 +1297,7 @@
       <c r="A34" s="13"/>
       <c r="B34" s="4"/>
       <c r="C34" s="20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D34" s="4"/>
       <c r="E34" s="11"/>
@@ -1315,7 +1310,7 @@
       <c r="B35" s="19"/>
       <c r="C35" s="19"/>
       <c r="D35" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E35" s="25"/>
       <c r="F35" s="30" t="b">
@@ -1327,7 +1322,7 @@
       <c r="B36" s="4"/>
       <c r="C36" s="22"/>
       <c r="D36" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E36" s="36"/>
       <c r="F36" s="31" t="b">
@@ -1339,7 +1334,7 @@
       <c r="B37" s="19"/>
       <c r="C37" s="19"/>
       <c r="D37" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E37" s="25"/>
       <c r="F37" s="30" t="b">
@@ -1351,7 +1346,7 @@
       <c r="B38" s="23"/>
       <c r="C38" s="23"/>
       <c r="D38" s="37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E38" s="25"/>
       <c r="F38" s="12" t="b">
@@ -1363,7 +1358,7 @@
       <c r="B39" s="23"/>
       <c r="C39" s="23"/>
       <c r="D39" s="28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E39" s="25"/>
       <c r="F39" s="12" t="b">
@@ -1374,7 +1369,7 @@
       <c r="A40" s="13"/>
       <c r="B40" s="4"/>
       <c r="C40" s="20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="11"/>
@@ -1387,7 +1382,7 @@
       <c r="B41" s="19"/>
       <c r="C41" s="19"/>
       <c r="D41" s="16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E41" s="25"/>
       <c r="F41" s="30" t="b">
@@ -1399,7 +1394,7 @@
       <c r="B42" s="4"/>
       <c r="C42" s="22"/>
       <c r="D42" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E42" s="36"/>
       <c r="F42" s="31" t="b">
@@ -1411,7 +1406,7 @@
       <c r="B43" s="19"/>
       <c r="C43" s="19"/>
       <c r="D43" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E43" s="25"/>
       <c r="F43" s="30" t="b">
@@ -1423,7 +1418,7 @@
       <c r="B44" s="19"/>
       <c r="C44" s="19"/>
       <c r="D44" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E44" s="25"/>
       <c r="F44" s="12" t="b">
@@ -1435,7 +1430,7 @@
       <c r="B45" s="19"/>
       <c r="C45" s="19"/>
       <c r="D45" s="16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E45" s="25"/>
       <c r="F45" s="12" t="b">
@@ -1447,7 +1442,7 @@
       <c r="B46" s="19"/>
       <c r="C46" s="19"/>
       <c r="D46" s="16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E46" s="25"/>
       <c r="F46" s="12" t="b">
@@ -1459,7 +1454,7 @@
       <c r="B47" s="19"/>
       <c r="C47" s="19"/>
       <c r="D47" s="16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E47" s="25"/>
       <c r="F47" s="12" t="b">
@@ -1469,11 +1464,11 @@
     <row r="48" ht="22.5" customHeight="1">
       <c r="A48" s="13"/>
       <c r="B48" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C48" s="15"/>
       <c r="D48" s="38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E48" s="39"/>
       <c r="F48" s="31" t="b">
@@ -1484,7 +1479,7 @@
       <c r="A49" s="22"/>
       <c r="B49" s="22"/>
       <c r="C49" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D49" s="4"/>
       <c r="E49" s="40"/>
@@ -1497,7 +1492,7 @@
       <c r="B50" s="22"/>
       <c r="C50" s="19"/>
       <c r="D50" s="16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E50" s="41"/>
       <c r="F50" s="24"/>
@@ -1507,10 +1502,10 @@
       <c r="B51" s="22"/>
       <c r="C51" s="22"/>
       <c r="D51" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="E51" s="32" t="s">
         <v>51</v>
-      </c>
-      <c r="E51" s="32" t="s">
-        <v>52</v>
       </c>
       <c r="F51" s="17" t="b">
         <v>0</v>
@@ -1521,7 +1516,7 @@
       <c r="B52" s="22"/>
       <c r="C52" s="19"/>
       <c r="D52" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E52" s="41"/>
       <c r="F52" s="31" t="b">
@@ -1533,7 +1528,7 @@
       <c r="B53" s="22"/>
       <c r="C53" s="23"/>
       <c r="D53" s="28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E53" s="28"/>
       <c r="F53" s="42" t="b">
@@ -1544,7 +1539,7 @@
       <c r="A54" s="27"/>
       <c r="B54" s="4"/>
       <c r="C54" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D54" s="4"/>
       <c r="E54" s="43"/>
@@ -1557,7 +1552,7 @@
       <c r="B55" s="19"/>
       <c r="C55" s="19"/>
       <c r="D55" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E55" s="36"/>
       <c r="F55" s="31" t="b">
@@ -1569,7 +1564,7 @@
       <c r="B56" s="4"/>
       <c r="C56" s="22"/>
       <c r="D56" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E56" s="25"/>
       <c r="F56" s="30" t="b">
@@ -1581,7 +1576,7 @@
       <c r="B57" s="19"/>
       <c r="C57" s="19"/>
       <c r="D57" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E57" s="36"/>
       <c r="F57" s="31" t="b">
@@ -1592,7 +1587,7 @@
       <c r="A58" s="27"/>
       <c r="B58" s="4"/>
       <c r="C58" s="20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D58" s="4"/>
       <c r="E58" s="43"/>
@@ -1605,7 +1600,7 @@
       <c r="B59" s="19"/>
       <c r="C59" s="19"/>
       <c r="D59" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E59" s="36"/>
       <c r="F59" s="31" t="b">
@@ -1617,7 +1612,7 @@
       <c r="B60" s="4"/>
       <c r="C60" s="22"/>
       <c r="D60" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E60" s="25"/>
       <c r="F60" s="30" t="b">
@@ -1629,7 +1624,7 @@
       <c r="B61" s="19"/>
       <c r="C61" s="19"/>
       <c r="D61" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E61" s="36"/>
       <c r="F61" s="31" t="b">
@@ -1640,7 +1635,7 @@
       <c r="A62" s="18"/>
       <c r="B62" s="19"/>
       <c r="C62" s="16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D62" s="16"/>
       <c r="E62" s="25"/>
@@ -1653,7 +1648,7 @@
       <c r="B63" s="19"/>
       <c r="C63" s="19"/>
       <c r="D63" s="16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E63" s="25"/>
       <c r="F63" s="26" t="b">
@@ -1664,7 +1659,7 @@
       <c r="A64" s="18"/>
       <c r="B64" s="19"/>
       <c r="C64" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D64" s="16"/>
       <c r="E64" s="25"/>
@@ -1677,7 +1672,7 @@
       <c r="B65" s="19"/>
       <c r="C65" s="19"/>
       <c r="D65" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E65" s="25"/>
       <c r="F65" s="26" t="b">
@@ -1689,7 +1684,7 @@
       <c r="B66" s="19"/>
       <c r="C66" s="19"/>
       <c r="D66" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E66" s="25"/>
       <c r="F66" s="26" t="b">
@@ -1700,7 +1695,7 @@
       <c r="A67" s="18"/>
       <c r="B67" s="19"/>
       <c r="C67" s="16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D67" s="16"/>
       <c r="E67" s="25"/>
@@ -1713,7 +1708,7 @@
       <c r="B68" s="19"/>
       <c r="C68" s="22"/>
       <c r="D68" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E68" s="25"/>
       <c r="F68" s="26" t="b">
@@ -1725,7 +1720,7 @@
       <c r="B69" s="19"/>
       <c r="C69" s="22"/>
       <c r="D69" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E69" s="25"/>
       <c r="F69" s="26" t="b">
@@ -1737,7 +1732,7 @@
       <c r="B70" s="19"/>
       <c r="C70" s="22"/>
       <c r="D70" s="16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E70" s="25"/>
       <c r="F70" s="26" t="b">
@@ -1749,7 +1744,7 @@
       <c r="B71" s="19"/>
       <c r="C71" s="19"/>
       <c r="D71" s="16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E71" s="25"/>
       <c r="F71" s="26" t="b">
@@ -1761,7 +1756,7 @@
       <c r="B72" s="19"/>
       <c r="C72" s="19"/>
       <c r="D72" s="16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E72" s="25"/>
       <c r="F72" s="26" t="b">
@@ -1772,7 +1767,7 @@
       <c r="A73" s="18"/>
       <c r="B73" s="19"/>
       <c r="C73" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D73" s="16"/>
       <c r="E73" s="25"/>
@@ -1813,11 +1808,11 @@
     <row r="77" ht="22.5" customHeight="1">
       <c r="A77" s="27"/>
       <c r="B77" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C77" s="15"/>
       <c r="D77" s="38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E77" s="29"/>
       <c r="F77" s="30" t="b">
@@ -1828,7 +1823,7 @@
       <c r="A78" s="13"/>
       <c r="B78" s="4"/>
       <c r="C78" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D78" s="4"/>
       <c r="E78" s="11"/>
@@ -1841,7 +1836,7 @@
       <c r="B79" s="19"/>
       <c r="C79" s="19"/>
       <c r="D79" s="16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E79" s="25"/>
       <c r="F79" s="30" t="b">
@@ -1853,7 +1848,7 @@
       <c r="B80" s="4"/>
       <c r="C80" s="22"/>
       <c r="D80" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E80" s="36"/>
       <c r="F80" s="31" t="b">
@@ -1865,7 +1860,7 @@
       <c r="B81" s="19"/>
       <c r="C81" s="19"/>
       <c r="D81" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E81" s="25"/>
       <c r="F81" s="30" t="b">
@@ -1876,7 +1871,7 @@
       <c r="A82" s="13"/>
       <c r="B82" s="4"/>
       <c r="C82" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D82" s="4"/>
       <c r="E82" s="11"/>
@@ -1889,7 +1884,7 @@
       <c r="B83" s="19"/>
       <c r="C83" s="19"/>
       <c r="D83" s="16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E83" s="25"/>
       <c r="F83" s="30" t="b">
@@ -1901,7 +1896,7 @@
       <c r="B84" s="4"/>
       <c r="C84" s="22"/>
       <c r="D84" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E84" s="36"/>
       <c r="F84" s="31" t="b">
@@ -1913,7 +1908,7 @@
       <c r="B85" s="19"/>
       <c r="C85" s="19"/>
       <c r="D85" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E85" s="25"/>
       <c r="F85" s="30" t="b">
@@ -1924,7 +1919,7 @@
       <c r="A86" s="13"/>
       <c r="B86" s="4"/>
       <c r="C86" s="20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D86" s="4"/>
       <c r="E86" s="11"/>
@@ -1937,7 +1932,7 @@
       <c r="B87" s="19"/>
       <c r="C87" s="19"/>
       <c r="D87" s="16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E87" s="25"/>
       <c r="F87" s="30" t="b">
@@ -1949,7 +1944,7 @@
       <c r="B88" s="4"/>
       <c r="C88" s="22"/>
       <c r="D88" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E88" s="36"/>
       <c r="F88" s="31" t="b">
@@ -1961,7 +1956,7 @@
       <c r="B89" s="19"/>
       <c r="C89" s="19"/>
       <c r="D89" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E89" s="25"/>
       <c r="F89" s="30" t="b">

</xml_diff>